<commit_message>
test: fixture workbooks without the folder Excel saved them in
Excel records the folder it saved a workbook in as x15ac:absPath, inside
an mc:AlternateContent block in xl/workbook.xml. 246 of the 254
committed fixture workbooks carried one: a temp folder, this checkout's
fixture folders, or pyOfficeEditor's.

scripts/strip_fixture_save_paths.py takes the block out of each through
the library's own package reader and writer. Every other part keeps its
bytes, header and compressed body alike, and each rewrite is checked
before it is written. The measurement scripts that save or copy a
workbook into tests/fixtures do the same through
scripts/fixture_workbook.py, so a new fixture comes in clean.

No test compares a scrubbed workbook.xml with Excel's bytes. The one
whole-package comparison, the untouched save of excel_shapes.xlsm,
compares the model's save with the fixture itself. The suite gives the
same counts before and after: 21,276 passed, 228 skipped, 65 xfailed.
</commit_message>
<xml_diff>
--- a/tests/fixtures/at_sign.xlsx
+++ b/tests/fixtures/at_sign.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\William\AppData\Local\Temp\tmpf1piv6vt\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{4D9D71E3-8FBD-4093-A0BE-497F4BEF1138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="7920" windowHeight="13995" xr2:uid="{7D3C4529-CD57-4674-99FD-E89739A1511B}"/>

</xml_diff>